<commit_message>
Add partial-quantity field for 副原料 and auto expiry-kind detection
- 副原料 records get a 半端量 (partial kg) input: whole amount and
  opened-package remainder are entered separately, the app sums them
  into 数量 and stores the breakdown in a new 半端量 column (workbook
  RecordTable is now 14 columns; seed regenerated)
- Entering 期限日 auto-selects 期限区分 by month distance from today
  (this month or earlier → 期限切れ, next → 来月期限, the one after →
  再来月期限, later → blank), still editable by hand
- Edit form decomposes a saved total back into whole + partial amounts;
  records list and CSV show the partial breakdown

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgvGiotwKBR4F3r5Tdot14
</commit_message>
<xml_diff>
--- a/inventory-app/data/inventory.xlsx
+++ b/inventory-app/data/inventory.xlsx
@@ -142,9 +142,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecordTable" displayName="RecordTable" ref="A1:M2" headerRowCount="1">
-  <autoFilter ref="A1:M2"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecordTable" displayName="RecordTable" ref="A1:N2" headerRowCount="1">
+  <autoFilter ref="A1:N2"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="記録ID"/>
     <tableColumn id="2" name="記録日時"/>
     <tableColumn id="3" name="棚卸し月"/>
@@ -153,11 +153,12 @@
     <tableColumn id="6" name="カテゴリ"/>
     <tableColumn id="7" name="数量"/>
     <tableColumn id="8" name="単位"/>
-    <tableColumn id="9" name="保管場所"/>
-    <tableColumn id="10" name="期限日"/>
-    <tableColumn id="11" name="期限区分"/>
-    <tableColumn id="12" name="入力者"/>
-    <tableColumn id="13" name="備考"/>
+    <tableColumn id="9" name="半端量"/>
+    <tableColumn id="10" name="保管場所"/>
+    <tableColumn id="11" name="期限日"/>
+    <tableColumn id="12" name="期限区分"/>
+    <tableColumn id="13" name="入力者"/>
+    <tableColumn id="14" name="備考"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -4371,7 +4372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4387,6 +4388,7 @@
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4432,25 +4434,30 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>半端量</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>保管場所</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>期限日</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>期限区分</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>入力者</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>備考</t>
         </is>

</xml_diff>

<commit_message>
Fix 半端量 semantics and add separate expired-stock fields
- 数量 is now entered as the total including 半端 (no auto-summing);
  半端量 is a breakdown memo of how much of that total is loose/odd,
  and the edit form shows both values back unchanged
- New 期限切れ量 / 期限切れ日 fields for 原料豆 and 副原料: expired
  stock is recorded separately from 数量, matching the paper sheet's
  「期限切れ（在庫合計に含まない）※期限も記入」 workflow
- RecordTable is now 16 columns (seed regenerated); records list and
  CSV show the expired amount and date

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgvGiotwKBR4F3r5Tdot14
</commit_message>
<xml_diff>
--- a/inventory-app/data/inventory.xlsx
+++ b/inventory-app/data/inventory.xlsx
@@ -142,9 +142,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecordTable" displayName="RecordTable" ref="A1:N2" headerRowCount="1">
-  <autoFilter ref="A1:N2"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecordTable" displayName="RecordTable" ref="A1:P2" headerRowCount="1">
+  <autoFilter ref="A1:P2"/>
+  <tableColumns count="16">
     <tableColumn id="1" name="記録ID"/>
     <tableColumn id="2" name="記録日時"/>
     <tableColumn id="3" name="棚卸し月"/>
@@ -154,11 +154,13 @@
     <tableColumn id="7" name="数量"/>
     <tableColumn id="8" name="単位"/>
     <tableColumn id="9" name="半端量"/>
-    <tableColumn id="10" name="保管場所"/>
-    <tableColumn id="11" name="期限日"/>
-    <tableColumn id="12" name="期限区分"/>
-    <tableColumn id="13" name="入力者"/>
-    <tableColumn id="14" name="備考"/>
+    <tableColumn id="10" name="期限切れ量"/>
+    <tableColumn id="11" name="期限切れ日"/>
+    <tableColumn id="12" name="保管場所"/>
+    <tableColumn id="13" name="期限日"/>
+    <tableColumn id="14" name="期限区分"/>
+    <tableColumn id="15" name="入力者"/>
+    <tableColumn id="16" name="備考"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -4372,7 +4374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4389,6 +4391,8 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4439,25 +4443,35 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>期限切れ量</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>期限切れ日</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>保管場所</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>期限日</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>期限区分</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>入力者</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>備考</t>
         </is>

</xml_diff>

<commit_message>
Add per-record double-check workflow and readable list chips
- Records now carry a check status (未確認 → 1回目完了 →
  ダブルチェック完了) with the double-checker's name and timestamp;
  new records default to 1回目完了. The edit sheet has a 3-state
  segmented control, and marking ダブルチェック完了 stamps the
  current member + JST time (reverting clears them)
- Records list: the cramped info line is now labeled chips
  (🕐 time / 👤 member / 半端 / ⚠ expired / 📍 location / ⏳ expiry),
  each row shows a color-coded status chip, and a progress summary
  (未確認 / 1回目完了 / ダブル済 counts) sits above the list
- RecordTable is now 19 columns (seed regenerated); CSV includes the
  three check columns

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgvGiotwKBR4F3r5Tdot14
</commit_message>
<xml_diff>
--- a/inventory-app/data/inventory.xlsx
+++ b/inventory-app/data/inventory.xlsx
@@ -142,9 +142,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecordTable" displayName="RecordTable" ref="A1:P2" headerRowCount="1">
-  <autoFilter ref="A1:P2"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecordTable" displayName="RecordTable" ref="A1:S2" headerRowCount="1">
+  <autoFilter ref="A1:S2"/>
+  <tableColumns count="19">
     <tableColumn id="1" name="記録ID"/>
     <tableColumn id="2" name="記録日時"/>
     <tableColumn id="3" name="棚卸し月"/>
@@ -160,7 +160,10 @@
     <tableColumn id="13" name="期限日"/>
     <tableColumn id="14" name="期限区分"/>
     <tableColumn id="15" name="入力者"/>
-    <tableColumn id="16" name="備考"/>
+    <tableColumn id="16" name="チェック状態"/>
+    <tableColumn id="17" name="ダブルチェック者"/>
+    <tableColumn id="18" name="ダブルチェック日時"/>
+    <tableColumn id="19" name="備考"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -4374,7 +4377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4393,6 +4396,9 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4472,6 +4478,21 @@
         </is>
       </c>
       <c r="P1" t="inlineStr">
+        <is>
+          <t>チェック状態</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>ダブルチェック者</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ダブルチェック日時</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>備考</t>
         </is>

</xml_diff>